<commit_message>
🤖 [Robô] Status atualizado automaticamente
</commit_message>
<xml_diff>
--- a/monitor_protocolos.xlsx
+++ b/monitor_protocolos.xlsx
@@ -1,132 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MicaelleVitoria\Downloads\Monitor protocolos\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{768258BF-4501-4015-A820-3A2830A1B51B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Santana de Parnaíba" sheetId="1" r:id="rId1"/>
-    <sheet name="Planilha1" sheetId="2" r:id="rId2"/>
+    <sheet name="Santana de Parnaíba" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Planilha1" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
-  <si>
-    <t>UNNAMED: 0</t>
-  </si>
-  <si>
-    <t>PROTOCOLO</t>
-  </si>
-  <si>
-    <t>REQUERIMENTO/DOCUMENTO</t>
-  </si>
-  <si>
-    <t>REQUERENTE/REMETENTE</t>
-  </si>
-  <si>
-    <t>PROPRIETÁRIO/DESTINATÁRIO</t>
-  </si>
-  <si>
-    <t>CRIADO EM</t>
-  </si>
-  <si>
-    <t>ÚLTIMA AÇÃO</t>
-  </si>
-  <si>
-    <t>STATUS ATUAL</t>
-  </si>
-  <si>
-    <t>ATIVO</t>
-  </si>
-  <si>
-    <t>MODIFICADO EM</t>
-  </si>
-  <si>
-    <t>668-26-PMSP-CUO</t>
-  </si>
-  <si>
-    <t>Certidão de Uso e Ocupação do Solo</t>
-  </si>
-  <si>
-    <t>Caroline Tiemi (caroline@artesanourbanismo.com.br)</t>
-  </si>
-  <si>
-    <t>MORRO AZUL EMPREENDIMENTOS IMOBILIÁRIOS LTDA.</t>
-  </si>
-  <si>
-    <t>26/03/2026</t>
-  </si>
-  <si>
-    <t>Ricardo Selli de Oliveira</t>
-  </si>
-  <si>
-    <t>SIM</t>
-  </si>
-  <si>
-    <t>26/05/2026 14:33</t>
-  </si>
-  <si>
-    <t>3163-25-PMSP-AUC</t>
-  </si>
-  <si>
-    <t>Processo encerrado por</t>
-  </si>
-  <si>
-    <t>NÃO</t>
-  </si>
-  <si>
-    <t>3040-25-PMSP-AUC</t>
-  </si>
-  <si>
-    <t>Testando robo</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -134,26 +45,94 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -441,104 +420,161 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="38" customWidth="1"/>
-    <col min="4" max="4" width="54" customWidth="1"/>
-    <col min="5" max="5" width="49" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="29" customWidth="1"/>
-    <col min="8" max="8" width="40" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="20" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>UNNAMED: 0</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>PROTOCOLO</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>REQUERIMENTO/DOCUMENTO</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>REQUERENTE/REMETENTE</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>PROPRIETÁRIO/DESTINATÁRIO</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>CRIADO EM</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>ÚLTIMA AÇÃO</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>STATUS ATUAL</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>MODIFICADO EM</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J2" t="s">
-        <v>17</v>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>668-26-PMSP-CUO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Certidão de Uso e Ocupação do Solo</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Caroline Tiemi (caroline@artesanourbanismo.com.br)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>MORRO AZUL EMPREENDIMENTOS IMOBILIÁRIOS LTDA.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>26/03/2026</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Ricardo Selli de Oliveira</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Processo encaminhado para Relatórios</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>28/05/2026 17:48:10</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3" t="s">
-        <v>19</v>
-      </c>
-      <c r="I3" t="s">
-        <v>20</v>
-      </c>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>3163-25-PMSP-AUC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Processo encerrado por</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B4" t="s">
-        <v>21</v>
-      </c>
-      <c r="H4" t="s">
-        <v>19</v>
-      </c>
-      <c r="I4" t="s">
-        <v>20</v>
-      </c>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3040-25-PMSP-AUC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Processo encerrado por</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -546,9 +582,13 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Atualização automática de status: 28/05/2026 19:17:06
</commit_message>
<xml_diff>
--- a/monitor_protocolos.xlsx
+++ b/monitor_protocolos.xlsx
@@ -1,129 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MicaelleVitoria\Downloads\Monitor protocolos\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6B3D7D2-ADA4-4616-8AFD-403B31A5D650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1656" yWindow="2412" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1656" yWindow="2412" windowWidth="17280" windowHeight="8880" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Santana de Parnaíba" sheetId="1" r:id="rId1"/>
-    <sheet name="Planilha1" sheetId="2" r:id="rId2"/>
+    <sheet name="Santana de Parnaíba" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Planilha1" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
-  <si>
-    <t>UNNAMED: 0</t>
-  </si>
-  <si>
-    <t>PROTOCOLO</t>
-  </si>
-  <si>
-    <t>REQUERIMENTO/DOCUMENTO</t>
-  </si>
-  <si>
-    <t>REQUERENTE/REMETENTE</t>
-  </si>
-  <si>
-    <t>PROPRIETÁRIO/DESTINATÁRIO</t>
-  </si>
-  <si>
-    <t>CRIADO EM</t>
-  </si>
-  <si>
-    <t>ÚLTIMA AÇÃO</t>
-  </si>
-  <si>
-    <t>STATUS ATUAL</t>
-  </si>
-  <si>
-    <t>ATIVO</t>
-  </si>
-  <si>
-    <t>MODIFICADO EM</t>
-  </si>
-  <si>
-    <t>668-26-PMSP-CUO</t>
-  </si>
-  <si>
-    <t>Certidão de Uso e Ocupação do Solo</t>
-  </si>
-  <si>
-    <t>Caroline Tiemi (caroline@artesanourbanismo.com.br)</t>
-  </si>
-  <si>
-    <t>MORRO AZUL EMPREENDIMENTOS IMOBILIÁRIOS LTDA.</t>
-  </si>
-  <si>
-    <t>26/03/2026</t>
-  </si>
-  <si>
-    <t>SIM</t>
-  </si>
-  <si>
-    <t>26/05/2026 14:33</t>
-  </si>
-  <si>
-    <t>3163-25-PMSP-AUC</t>
-  </si>
-  <si>
-    <t>Processo encerrado por</t>
-  </si>
-  <si>
-    <t>NÃO</t>
-  </si>
-  <si>
-    <t>3040-25-PMSP-AUC</t>
-  </si>
-  <si>
-    <t>TESTE</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -131,26 +45,94 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -438,101 +420,157 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="38" customWidth="1"/>
-    <col min="4" max="4" width="54" customWidth="1"/>
-    <col min="5" max="5" width="49" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="29" customWidth="1"/>
-    <col min="8" max="8" width="40" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="20" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>UNNAMED: 0</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>PROTOCOLO</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>REQUERIMENTO/DOCUMENTO</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>REQUERENTE/REMETENTE</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>PROPRIETÁRIO/DESTINATÁRIO</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>CRIADO EM</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>ÚLTIMA AÇÃO</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>STATUS ATUAL</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>MODIFICADO EM</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I2" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" t="s">
-        <v>16</v>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>668-26-PMSP-CUO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Certidão de Uso e Ocupação do Solo</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Caroline Tiemi (caroline@artesanourbanismo.com.br)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>MORRO AZUL EMPREENDIMENTOS IMOBILIÁRIOS LTDA.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>26/03/2026</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Processo encaminhado para Relatórios</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>28/05/2026 19:17:06</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I3" t="s">
-        <v>19</v>
-      </c>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>3163-25-PMSP-AUC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Processo encerrado por</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I4" t="s">
-        <v>19</v>
-      </c>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3040-25-PMSP-AUC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Processo encerrado por</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -540,9 +578,13 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Substituição total de linhas alteradas: 29/05/2026 14:31:22
</commit_message>
<xml_diff>
--- a/monitor_protocolos.xlsx
+++ b/monitor_protocolos.xlsx
@@ -1,134 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://artesanourbanismo-my.sharepoint.com/personal/mvitoria_artesanourbanismo_com_br/Documents/Monitor protocolos/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{6D3BE9E3-B4C0-47EB-8398-2B17DC85FF49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B1C58B7-EEAB-40B9-9C08-6BE36876EB94}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-1575" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-1575" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Santana de Parnaíba" sheetId="1" r:id="rId1"/>
+    <sheet name="Santana de Parnaíba" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
-  <si>
-    <t>UNNAMED: 0</t>
-  </si>
-  <si>
-    <t>PROTOCOLO</t>
-  </si>
-  <si>
-    <t>REQUERIMENTO/DOCUMENTO</t>
-  </si>
-  <si>
-    <t>REQUERENTE/REMETENTE</t>
-  </si>
-  <si>
-    <t>PROPRIETÁRIO/DESTINATÁRIO</t>
-  </si>
-  <si>
-    <t>CRIADO EM</t>
-  </si>
-  <si>
-    <t>ÚLTIMA AÇÃO</t>
-  </si>
-  <si>
-    <t>STATUS ATUAL</t>
-  </si>
-  <si>
-    <t>ATIVO</t>
-  </si>
-  <si>
-    <t>MODIFICADO EM</t>
-  </si>
-  <si>
-    <t>668-26-PMSP-CUO</t>
-  </si>
-  <si>
-    <t>Certidão de Uso e Ocupação do Solo</t>
-  </si>
-  <si>
-    <t>Caroline Tiemi (caroline@artesanourbanismo.com.br)</t>
-  </si>
-  <si>
-    <t>MORRO AZUL EMPREENDIMENTOS IMOBILIÁRIOS LTDA.</t>
-  </si>
-  <si>
-    <t>26/03/2026</t>
-  </si>
-  <si>
-    <t>Ricardo Selli de Oliveira</t>
-  </si>
-  <si>
-    <t>SIM</t>
-  </si>
-  <si>
-    <t>26/05/2026 14:17</t>
-  </si>
-  <si>
-    <t>3163-25-PMSP-AUC</t>
-  </si>
-  <si>
-    <t>Processo encerrado por</t>
-  </si>
-  <si>
-    <t>NÃO</t>
-  </si>
-  <si>
-    <t>3040-25-PMSP-AUC</t>
-  </si>
-  <si>
-    <t>Processo</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -136,14 +44,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -151,38 +68,79 @@
   </cellStyles>
   <dxfs count="1">
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="bottom"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FB1F5021-ED65-41CF-8087-F798A92E5D17}" name="Tabela1" displayName="Tabela1" ref="A1:J4" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:J4" xr:uid="{FB1F5021-ED65-41CF-8087-F798A92E5D17}"/>
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{8C0E23F6-EA0F-47FE-93AA-74BA6595A85B}" name="UNNAMED: 0"/>
-    <tableColumn id="2" xr3:uid="{9114CD1F-C9E2-4B73-ADAE-B1190218C286}" name="PROTOCOLO"/>
-    <tableColumn id="3" xr3:uid="{EE2C434F-DBF6-4E89-9514-EAFD75A1D7E2}" name="REQUERIMENTO/DOCUMENTO"/>
-    <tableColumn id="4" xr3:uid="{B7482B76-6A04-4537-9429-222BB7420E80}" name="REQUERENTE/REMETENTE"/>
-    <tableColumn id="5" xr3:uid="{10240438-31ED-4523-A4E7-31F7DEBCC8D8}" name="PROPRIETÁRIO/DESTINATÁRIO"/>
-    <tableColumn id="6" xr3:uid="{9BFD0E9D-85BC-47FA-B8E1-ACDD792AA995}" name="CRIADO EM"/>
-    <tableColumn id="7" xr3:uid="{D289B279-DFFC-4A26-A3EF-007414E7A55D}" name="ÚLTIMA AÇÃO"/>
-    <tableColumn id="8" xr3:uid="{E0901626-3F1A-4C9D-ABEC-EDF33995EA74}" name="STATUS ATUAL"/>
-    <tableColumn id="9" xr3:uid="{6C9A014B-F705-44ED-BF42-1314E3FB83E7}" name="ATIVO"/>
-    <tableColumn id="10" xr3:uid="{F1C9B428-05B8-4134-810D-9C876DC897D7}" name="MODIFICADO EM"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight13" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -469,109 +427,147 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="38" customWidth="1"/>
-    <col min="4" max="4" width="54" customWidth="1"/>
-    <col min="5" max="5" width="49" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="29" customWidth="1"/>
-    <col min="8" max="8" width="40" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="20" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>UNNAMED: 0</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>PROTOCOLO</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>REQUERIMENTO/DOCUMENTO</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>REQUERENTE/REMETENTE</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>PROPRIETÁRIO/DESTINATÁRIO</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>CRIADO EM</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>ÚLTIMA AÇÃO</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>STATUS ATUAL</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>MODIFICADO EM</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J2" t="s">
-        <v>17</v>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>668-26-PMSP-CUO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Processo encaminhado para Relatórios</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>29/05/2026 14:31:22</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I3" t="s">
-        <v>16</v>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>3163-25-PMSP-AUC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Processo encerrado por deferimento</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>29/05/2026 14:31:22</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B4" t="s">
-        <v>21</v>
-      </c>
-      <c r="H4" t="s">
-        <v>19</v>
-      </c>
-      <c r="I4" t="s">
-        <v>20</v>
-      </c>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3040-25-PMSP-AUC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Processo encerrado por</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
🤖 Substituição total de linhas alteradas: 29/05/2026 14:48:55
</commit_message>
<xml_diff>
--- a/monitor_protocolos.xlsx
+++ b/monitor_protocolos.xlsx
@@ -1,134 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://artesanourbanismo-my.sharepoint.com/personal/mvitoria_artesanourbanismo_com_br/Documents/Monitor protocolos/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{6D3BE9E3-B4C0-47EB-8398-2B17DC85FF49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E323891D-8704-488C-9FCD-C066432A1C93}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-1575" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-1575" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Santana de Parnaíba" sheetId="1" r:id="rId1"/>
+    <sheet name="Santana de Parnaíba" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
-  <si>
-    <t>UNNAMED: 0</t>
-  </si>
-  <si>
-    <t>PROTOCOLO</t>
-  </si>
-  <si>
-    <t>REQUERIMENTO/DOCUMENTO</t>
-  </si>
-  <si>
-    <t>REQUERENTE/REMETENTE</t>
-  </si>
-  <si>
-    <t>PROPRIETÁRIO/DESTINATÁRIO</t>
-  </si>
-  <si>
-    <t>CRIADO EM</t>
-  </si>
-  <si>
-    <t>ÚLTIMA AÇÃO</t>
-  </si>
-  <si>
-    <t>STATUS ATUAL</t>
-  </si>
-  <si>
-    <t>ATIVO</t>
-  </si>
-  <si>
-    <t>MODIFICADO EM</t>
-  </si>
-  <si>
-    <t>668-26-PMSP-CUO</t>
-  </si>
-  <si>
-    <t>Certidão de Uso e Ocupação do Solo</t>
-  </si>
-  <si>
-    <t>Caroline Tiemi (caroline@artesanourbanismo.com.br)</t>
-  </si>
-  <si>
-    <t>MORRO AZUL EMPREENDIMENTOS IMOBILIÁRIOS LTDA.</t>
-  </si>
-  <si>
-    <t>26/03/2026</t>
-  </si>
-  <si>
-    <t>SIM</t>
-  </si>
-  <si>
-    <t>26/05/2026 14:17</t>
-  </si>
-  <si>
-    <t>3163-25-PMSP-AUC</t>
-  </si>
-  <si>
-    <t>Processo encerrado por</t>
-  </si>
-  <si>
-    <t>NÃO</t>
-  </si>
-  <si>
-    <t>3040-25-PMSP-AUC</t>
-  </si>
-  <si>
-    <t>Ricardo</t>
-  </si>
-  <si>
-    <t>Process</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -136,14 +44,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -151,38 +68,79 @@
   </cellStyles>
   <dxfs count="1">
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="bottom"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FB1F5021-ED65-41CF-8087-F798A92E5D17}" name="Tabela1" displayName="Tabela1" ref="A1:J4" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:J4" xr:uid="{FB1F5021-ED65-41CF-8087-F798A92E5D17}"/>
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{8C0E23F6-EA0F-47FE-93AA-74BA6595A85B}" name="UNNAMED: 0"/>
-    <tableColumn id="2" xr3:uid="{9114CD1F-C9E2-4B73-ADAE-B1190218C286}" name="PROTOCOLO"/>
-    <tableColumn id="3" xr3:uid="{EE2C434F-DBF6-4E89-9514-EAFD75A1D7E2}" name="REQUERIMENTO/DOCUMENTO"/>
-    <tableColumn id="4" xr3:uid="{B7482B76-6A04-4537-9429-222BB7420E80}" name="REQUERENTE/REMETENTE"/>
-    <tableColumn id="5" xr3:uid="{10240438-31ED-4523-A4E7-31F7DEBCC8D8}" name="PROPRIETÁRIO/DESTINATÁRIO"/>
-    <tableColumn id="6" xr3:uid="{9BFD0E9D-85BC-47FA-B8E1-ACDD792AA995}" name="CRIADO EM"/>
-    <tableColumn id="7" xr3:uid="{D289B279-DFFC-4A26-A3EF-007414E7A55D}" name="ÚLTIMA AÇÃO"/>
-    <tableColumn id="8" xr3:uid="{E0901626-3F1A-4C9D-ABEC-EDF33995EA74}" name="STATUS ATUAL"/>
-    <tableColumn id="9" xr3:uid="{6C9A014B-F705-44ED-BF42-1314E3FB83E7}" name="ATIVO"/>
-    <tableColumn id="10" xr3:uid="{F1C9B428-05B8-4134-810D-9C876DC897D7}" name="MODIFICADO EM"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight13" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -469,109 +427,147 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="38" customWidth="1"/>
-    <col min="4" max="4" width="54" customWidth="1"/>
-    <col min="5" max="5" width="49" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="29" customWidth="1"/>
-    <col min="8" max="8" width="40" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="20" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>UNNAMED: 0</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>PROTOCOLO</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>REQUERIMENTO/DOCUMENTO</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>REQUERENTE/REMETENTE</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>PROPRIETÁRIO/DESTINATÁRIO</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>CRIADO EM</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>ÚLTIMA AÇÃO</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>STATUS ATUAL</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>MODIFICADO EM</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I2" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" t="s">
-        <v>16</v>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>668-26-PMSP-CUO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Processo encaminhado para Relatórios</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>29/05/2026 14:48:55</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I3" t="s">
-        <v>15</v>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>3163-25-PMSP-AUC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Processo encerrado por deferimento</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>29/05/2026 14:48:55</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I4" t="s">
-        <v>19</v>
-      </c>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3040-25-PMSP-AUC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Processo encerrado por</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
🤖 Substituição total de linhas alteradas: 29/05/2026 14:58:46
</commit_message>
<xml_diff>
--- a/monitor_protocolos.xlsx
+++ b/monitor_protocolos.xlsx
@@ -1,134 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://artesanourbanismo-my.sharepoint.com/personal/mvitoria_artesanourbanismo_com_br/Documents/Monitor protocolos/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{6D3BE9E3-B4C0-47EB-8398-2B17DC85FF49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E323891D-8704-488C-9FCD-C066432A1C93}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-1575" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-1575" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Santana de Parnaíba" sheetId="1" r:id="rId1"/>
+    <sheet name="Santana de Parnaíba" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
-  <si>
-    <t>UNNAMED: 0</t>
-  </si>
-  <si>
-    <t>PROTOCOLO</t>
-  </si>
-  <si>
-    <t>REQUERIMENTO/DOCUMENTO</t>
-  </si>
-  <si>
-    <t>REQUERENTE/REMETENTE</t>
-  </si>
-  <si>
-    <t>PROPRIETÁRIO/DESTINATÁRIO</t>
-  </si>
-  <si>
-    <t>CRIADO EM</t>
-  </si>
-  <si>
-    <t>ÚLTIMA AÇÃO</t>
-  </si>
-  <si>
-    <t>STATUS ATUAL</t>
-  </si>
-  <si>
-    <t>ATIVO</t>
-  </si>
-  <si>
-    <t>MODIFICADO EM</t>
-  </si>
-  <si>
-    <t>668-26-PMSP-CUO</t>
-  </si>
-  <si>
-    <t>Certidão de Uso e Ocupação do Solo</t>
-  </si>
-  <si>
-    <t>Caroline Tiemi (caroline@artesanourbanismo.com.br)</t>
-  </si>
-  <si>
-    <t>MORRO AZUL EMPREENDIMENTOS IMOBILIÁRIOS LTDA.</t>
-  </si>
-  <si>
-    <t>26/03/2026</t>
-  </si>
-  <si>
-    <t>SIM</t>
-  </si>
-  <si>
-    <t>26/05/2026 14:17</t>
-  </si>
-  <si>
-    <t>3163-25-PMSP-AUC</t>
-  </si>
-  <si>
-    <t>Processo encerrado por</t>
-  </si>
-  <si>
-    <t>NÃO</t>
-  </si>
-  <si>
-    <t>3040-25-PMSP-AUC</t>
-  </si>
-  <si>
-    <t>Ricardo</t>
-  </si>
-  <si>
-    <t>Process</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -136,14 +44,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -151,38 +68,79 @@
   </cellStyles>
   <dxfs count="1">
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="bottom"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FB1F5021-ED65-41CF-8087-F798A92E5D17}" name="Tabela1" displayName="Tabela1" ref="A1:J4" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:J4" xr:uid="{FB1F5021-ED65-41CF-8087-F798A92E5D17}"/>
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{8C0E23F6-EA0F-47FE-93AA-74BA6595A85B}" name="UNNAMED: 0"/>
-    <tableColumn id="2" xr3:uid="{9114CD1F-C9E2-4B73-ADAE-B1190218C286}" name="PROTOCOLO"/>
-    <tableColumn id="3" xr3:uid="{EE2C434F-DBF6-4E89-9514-EAFD75A1D7E2}" name="REQUERIMENTO/DOCUMENTO"/>
-    <tableColumn id="4" xr3:uid="{B7482B76-6A04-4537-9429-222BB7420E80}" name="REQUERENTE/REMETENTE"/>
-    <tableColumn id="5" xr3:uid="{10240438-31ED-4523-A4E7-31F7DEBCC8D8}" name="PROPRIETÁRIO/DESTINATÁRIO"/>
-    <tableColumn id="6" xr3:uid="{9BFD0E9D-85BC-47FA-B8E1-ACDD792AA995}" name="CRIADO EM"/>
-    <tableColumn id="7" xr3:uid="{D289B279-DFFC-4A26-A3EF-007414E7A55D}" name="ÚLTIMA AÇÃO"/>
-    <tableColumn id="8" xr3:uid="{E0901626-3F1A-4C9D-ABEC-EDF33995EA74}" name="STATUS ATUAL"/>
-    <tableColumn id="9" xr3:uid="{6C9A014B-F705-44ED-BF42-1314E3FB83E7}" name="ATIVO"/>
-    <tableColumn id="10" xr3:uid="{F1C9B428-05B8-4134-810D-9C876DC897D7}" name="MODIFICADO EM"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight13" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -469,109 +427,147 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="38" customWidth="1"/>
-    <col min="4" max="4" width="54" customWidth="1"/>
-    <col min="5" max="5" width="49" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="29" customWidth="1"/>
-    <col min="8" max="8" width="40" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="20" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>UNNAMED: 0</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>PROTOCOLO</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>REQUERIMENTO/DOCUMENTO</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>REQUERENTE/REMETENTE</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>PROPRIETÁRIO/DESTINATÁRIO</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>CRIADO EM</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>ÚLTIMA AÇÃO</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>STATUS ATUAL</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>MODIFICADO EM</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I2" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" t="s">
-        <v>16</v>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>668-26-PMSP-CUO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Processo encaminhado para Relatórios</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>29/05/2026 14:58:46</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I3" t="s">
-        <v>15</v>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>3163-25-PMSP-AUC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Processo encerrado por deferimento</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>29/05/2026 14:58:46</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I4" t="s">
-        <v>19</v>
-      </c>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3040-25-PMSP-AUC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Processo encerrado por</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>